<commit_message>
data: cierre dia 2026-08-17_1937 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/Stock/stock.xlsx
+++ b/01_INPUTS/Stock/stock.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47B1685F-5EB5-46B4-A07A-96584604963A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6FCEAC3-0A9F-4A2B-BC23-445767BC362F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2876,7 +2876,7 @@
         <v>24</v>
       </c>
       <c r="I2">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J2">
         <v>90</v>
@@ -2885,13 +2885,13 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -3212,7 +3212,7 @@
         <v>24</v>
       </c>
       <c r="I8">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="J8">
         <v>520</v>
@@ -3221,13 +3221,13 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O8">
         <v>0</v>
@@ -3660,7 +3660,7 @@
         <v>24</v>
       </c>
       <c r="I16">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J16">
         <v>116</v>
@@ -3669,13 +3669,13 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
       <c r="N16">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="O16">
         <v>0</v>
@@ -3884,16 +3884,16 @@
         <v>24</v>
       </c>
       <c r="I20">
-        <v>277</v>
+        <v>157</v>
       </c>
       <c r="J20">
-        <v>277</v>
+        <v>157</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>277</v>
+        <v>157</v>
       </c>
       <c r="M20">
         <v>0</v>
@@ -3940,7 +3940,7 @@
         <v>24</v>
       </c>
       <c r="I21">
-        <v>1113</v>
+        <v>1101</v>
       </c>
       <c r="J21">
         <v>1113</v>
@@ -3949,13 +3949,13 @@
         <v>0</v>
       </c>
       <c r="L21">
-        <v>1113</v>
+        <v>1101</v>
       </c>
       <c r="M21">
         <v>0</v>
       </c>
       <c r="N21">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O21">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         <v>24</v>
       </c>
       <c r="I22">
-        <v>413</v>
+        <v>371</v>
       </c>
       <c r="J22">
         <v>425</v>
@@ -4005,13 +4005,13 @@
         <v>0</v>
       </c>
       <c r="L22">
-        <v>413</v>
+        <v>371</v>
       </c>
       <c r="M22">
         <v>0</v>
       </c>
       <c r="N22">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="O22">
         <v>0</v>
@@ -4052,7 +4052,7 @@
         <v>24</v>
       </c>
       <c r="I23">
-        <v>2860</v>
+        <v>2686</v>
       </c>
       <c r="J23">
         <v>2866</v>
@@ -4061,13 +4061,13 @@
         <v>0</v>
       </c>
       <c r="L23">
-        <v>2860</v>
+        <v>2686</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <v>6</v>
+        <v>180</v>
       </c>
       <c r="O23">
         <v>0</v>
@@ -4108,7 +4108,7 @@
         <v>24</v>
       </c>
       <c r="I24">
-        <v>1410</v>
+        <v>1398</v>
       </c>
       <c r="J24">
         <v>1590</v>
@@ -4117,13 +4117,13 @@
         <v>0</v>
       </c>
       <c r="L24">
-        <v>1410</v>
+        <v>1398</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="O24">
         <v>0</v>
@@ -4780,7 +4780,7 @@
         <v>24</v>
       </c>
       <c r="I36">
-        <v>2128</v>
+        <v>2008</v>
       </c>
       <c r="J36">
         <v>2128</v>
@@ -4789,13 +4789,13 @@
         <v>0</v>
       </c>
       <c r="L36">
-        <v>2128</v>
+        <v>2008</v>
       </c>
       <c r="M36">
         <v>0</v>
       </c>
       <c r="N36">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="O36">
         <v>0</v>
@@ -5004,7 +5004,7 @@
         <v>24</v>
       </c>
       <c r="I40">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="J40">
         <v>54</v>
@@ -5013,13 +5013,13 @@
         <v>0</v>
       </c>
       <c r="L40">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="M40">
         <v>0</v>
       </c>
       <c r="N40">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O40">
         <v>0</v>
@@ -5228,7 +5228,7 @@
         <v>24</v>
       </c>
       <c r="I44">
-        <v>1221</v>
+        <v>1155</v>
       </c>
       <c r="J44">
         <v>1437</v>
@@ -5237,13 +5237,13 @@
         <v>0</v>
       </c>
       <c r="L44">
-        <v>1221</v>
+        <v>1155</v>
       </c>
       <c r="M44">
         <v>0</v>
       </c>
       <c r="N44">
-        <v>216</v>
+        <v>282</v>
       </c>
       <c r="O44">
         <v>0</v>
@@ -5284,7 +5284,7 @@
         <v>24</v>
       </c>
       <c r="I45">
-        <v>644</v>
+        <v>578</v>
       </c>
       <c r="J45">
         <v>1076</v>
@@ -5293,13 +5293,13 @@
         <v>0</v>
       </c>
       <c r="L45">
-        <v>644</v>
+        <v>578</v>
       </c>
       <c r="M45">
         <v>0</v>
       </c>
       <c r="N45">
-        <v>432</v>
+        <v>498</v>
       </c>
       <c r="O45">
         <v>0</v>
@@ -5508,7 +5508,7 @@
         <v>24</v>
       </c>
       <c r="I49">
-        <v>1827</v>
+        <v>1821</v>
       </c>
       <c r="J49">
         <v>1923</v>
@@ -5517,13 +5517,13 @@
         <v>0</v>
       </c>
       <c r="L49">
-        <v>1827</v>
+        <v>1821</v>
       </c>
       <c r="M49">
         <v>0</v>
       </c>
       <c r="N49">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="O49">
         <v>0</v>
@@ -6012,7 +6012,7 @@
         <v>24</v>
       </c>
       <c r="I58">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="J58">
         <v>120</v>
@@ -6021,13 +6021,13 @@
         <v>0</v>
       </c>
       <c r="L58">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="M58">
         <v>0</v>
       </c>
       <c r="N58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O58">
         <v>0</v>
@@ -6852,7 +6852,7 @@
         <v>24</v>
       </c>
       <c r="I73">
-        <v>1144</v>
+        <v>1138</v>
       </c>
       <c r="J73">
         <v>1144</v>
@@ -6861,13 +6861,13 @@
         <v>0</v>
       </c>
       <c r="L73">
-        <v>1144</v>
+        <v>1138</v>
       </c>
       <c r="M73">
         <v>0</v>
       </c>
       <c r="N73">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O73">
         <v>0</v>
@@ -6964,7 +6964,7 @@
         <v>24</v>
       </c>
       <c r="I75">
-        <v>651</v>
+        <v>645</v>
       </c>
       <c r="J75">
         <v>657</v>
@@ -6973,13 +6973,13 @@
         <v>0</v>
       </c>
       <c r="L75">
-        <v>651</v>
+        <v>645</v>
       </c>
       <c r="M75">
         <v>0</v>
       </c>
       <c r="N75">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="O75">
         <v>0</v>
@@ -7076,22 +7076,22 @@
         <v>24</v>
       </c>
       <c r="I77">
-        <v>1670</v>
+        <v>1658</v>
       </c>
       <c r="J77">
-        <v>1670</v>
+        <v>1664</v>
       </c>
       <c r="K77">
         <v>0</v>
       </c>
       <c r="L77">
-        <v>1670</v>
+        <v>1658</v>
       </c>
       <c r="M77">
         <v>0</v>
       </c>
       <c r="N77">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O77">
         <v>0</v>
@@ -7692,7 +7692,7 @@
         <v>24</v>
       </c>
       <c r="I88">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="J88">
         <v>276</v>
@@ -7701,13 +7701,13 @@
         <v>0</v>
       </c>
       <c r="L88">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="M88">
         <v>0</v>
       </c>
       <c r="N88">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O88">
         <v>0</v>
@@ -7860,7 +7860,7 @@
         <v>24</v>
       </c>
       <c r="I91">
-        <v>3863</v>
+        <v>3851</v>
       </c>
       <c r="J91">
         <v>4043</v>
@@ -7869,13 +7869,13 @@
         <v>0</v>
       </c>
       <c r="L91">
-        <v>3863</v>
+        <v>3851</v>
       </c>
       <c r="M91">
         <v>0</v>
       </c>
       <c r="N91">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="O91">
         <v>0</v>
@@ -8084,7 +8084,7 @@
         <v>24</v>
       </c>
       <c r="I95">
-        <v>813</v>
+        <v>807</v>
       </c>
       <c r="J95">
         <v>813</v>
@@ -8093,13 +8093,13 @@
         <v>0</v>
       </c>
       <c r="L95">
-        <v>813</v>
+        <v>807</v>
       </c>
       <c r="M95">
         <v>0</v>
       </c>
       <c r="N95">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O95">
         <v>0</v>
@@ -8196,7 +8196,7 @@
         <v>24</v>
       </c>
       <c r="I97">
-        <v>2565</v>
+        <v>2559</v>
       </c>
       <c r="J97">
         <v>2565</v>
@@ -8205,13 +8205,13 @@
         <v>0</v>
       </c>
       <c r="L97">
-        <v>2565</v>
+        <v>2559</v>
       </c>
       <c r="M97">
         <v>0</v>
       </c>
       <c r="N97">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O97">
         <v>0</v>
@@ -8924,7 +8924,7 @@
         <v>24</v>
       </c>
       <c r="I110">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="J110">
         <v>114</v>
@@ -8933,13 +8933,13 @@
         <v>0</v>
       </c>
       <c r="L110">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M110">
         <v>0</v>
       </c>
       <c r="N110">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O110">
         <v>0</v>
@@ -10324,7 +10324,7 @@
         <v>24</v>
       </c>
       <c r="I135">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="J135">
         <v>27</v>
@@ -10333,13 +10333,13 @@
         <v>0</v>
       </c>
       <c r="L135">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="M135">
         <v>0</v>
       </c>
       <c r="N135">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O135">
         <v>0</v>
@@ -10380,22 +10380,22 @@
         <v>24</v>
       </c>
       <c r="I136">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="J136">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="K136">
         <v>0</v>
       </c>
       <c r="L136">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="M136">
         <v>0</v>
       </c>
       <c r="N136">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O136">
         <v>0</v>
@@ -11388,7 +11388,7 @@
         <v>24</v>
       </c>
       <c r="I154">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J154">
         <v>27</v>
@@ -11397,13 +11397,13 @@
         <v>0</v>
       </c>
       <c r="L154">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="M154">
         <v>0</v>
       </c>
       <c r="N154">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O154">
         <v>0</v>
@@ -12116,7 +12116,7 @@
         <v>24</v>
       </c>
       <c r="I167">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="J167">
         <v>763</v>
@@ -12125,13 +12125,13 @@
         <v>0</v>
       </c>
       <c r="L167">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="M167">
         <v>0</v>
       </c>
       <c r="N167">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="O167">
         <v>0</v>
@@ -13121,7 +13121,7 @@
         <v>24</v>
       </c>
       <c r="I185">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="J185">
         <v>288</v>
@@ -13130,13 +13130,13 @@
         <v>0</v>
       </c>
       <c r="L185">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="M185">
         <v>0</v>
       </c>
       <c r="N185">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O185">
         <v>0</v>
@@ -13230,7 +13230,7 @@
         <v>24</v>
       </c>
       <c r="I187">
-        <v>1176</v>
+        <v>1164</v>
       </c>
       <c r="J187">
         <v>1182</v>
@@ -13239,13 +13239,13 @@
         <v>0</v>
       </c>
       <c r="L187">
-        <v>1176</v>
+        <v>1164</v>
       </c>
       <c r="M187">
         <v>0</v>
       </c>
       <c r="N187">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="O187">
         <v>0</v>
@@ -13566,7 +13566,7 @@
         <v>24</v>
       </c>
       <c r="I193">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="J193">
         <v>726</v>
@@ -13575,13 +13575,13 @@
         <v>0</v>
       </c>
       <c r="L193">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="M193">
         <v>0</v>
       </c>
       <c r="N193">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O193">
         <v>0</v>
@@ -13678,7 +13678,7 @@
         <v>24</v>
       </c>
       <c r="I195">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="J195">
         <v>894</v>
@@ -13687,13 +13687,13 @@
         <v>0</v>
       </c>
       <c r="L195">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="M195">
         <v>0</v>
       </c>
       <c r="N195">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O195">
         <v>0</v>
@@ -13902,7 +13902,7 @@
         <v>24</v>
       </c>
       <c r="I199">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="J199">
         <v>261</v>
@@ -13911,13 +13911,13 @@
         <v>0</v>
       </c>
       <c r="L199">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="M199">
         <v>0</v>
       </c>
       <c r="N199">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O199">
         <v>0</v>
@@ -14070,7 +14070,7 @@
         <v>24</v>
       </c>
       <c r="I202">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="J202">
         <v>480</v>
@@ -14079,13 +14079,13 @@
         <v>0</v>
       </c>
       <c r="L202">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="M202">
         <v>0</v>
       </c>
       <c r="N202">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="O202">
         <v>0</v>
@@ -14574,7 +14574,7 @@
         <v>24</v>
       </c>
       <c r="I211">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="J211">
         <v>402</v>
@@ -14583,13 +14583,13 @@
         <v>0</v>
       </c>
       <c r="L211">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="M211">
         <v>0</v>
       </c>
       <c r="N211">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O211">
         <v>0</v>
@@ -14686,22 +14686,22 @@
         <v>24</v>
       </c>
       <c r="I213">
-        <v>1809</v>
+        <v>1119</v>
       </c>
       <c r="J213">
-        <v>1812</v>
+        <v>1152</v>
       </c>
       <c r="K213">
         <v>0</v>
       </c>
       <c r="L213">
-        <v>1809</v>
+        <v>1119</v>
       </c>
       <c r="M213">
         <v>0</v>
       </c>
       <c r="N213">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="O213">
         <v>0</v>

</xml_diff>